<commit_message>
docs(reports): deploy unified consolidated summary reports for build 28
</commit_message>
<xml_diff>
--- a/reports/history/web/build-28/Excel/Passed_Test_Cases.xlsx
+++ b/reports/history/web/build-28/Excel/Passed_Test_Cases.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>15.23</t>
+          <t>13.72</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:01</t>
+          <t>2026-06-24 09:19:59</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr"/>
@@ -596,7 +596,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>5.63</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:07</t>
+          <t>2026-06-24 09:20:06</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
@@ -634,7 +634,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>4.43</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:12</t>
+          <t>2026-06-24 09:20:11</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr"/>
@@ -672,7 +672,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>4.44</t>
+          <t>5.06</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:16</t>
+          <t>2026-06-24 09:20:16</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
@@ -710,7 +710,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>9.78</t>
+          <t>9.83</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:21</t>
+          <t>2026-06-24 09:20:21</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
@@ -748,7 +748,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>5.67</t>
+          <t>6.03</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:31</t>
+          <t>2026-06-24 09:20:31</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr"/>
@@ -786,7 +786,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>3.37</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:36</t>
+          <t>2026-06-24 09:20:37</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr"/>
@@ -834,7 +834,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr"/>
@@ -872,7 +872,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr"/>
@@ -910,7 +910,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr"/>
@@ -986,7 +986,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr"/>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr"/>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr"/>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr"/>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr"/>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
@@ -1328,7 +1328,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
@@ -1404,7 +1404,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
@@ -1518,7 +1518,7 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
@@ -1594,7 +1594,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="G42" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:40</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
@@ -2278,7 +2278,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr"/>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H51" s="4" t="inlineStr"/>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr"/>
@@ -2430,7 +2430,7 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr"/>
@@ -2468,7 +2468,7 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr"/>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H55" s="4" t="inlineStr"/>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr"/>
@@ -2582,7 +2582,7 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H57" s="4" t="inlineStr"/>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr"/>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="G59" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H59" s="4" t="inlineStr"/>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr"/>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H61" s="4" t="inlineStr"/>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr"/>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H63" s="4" t="inlineStr"/>
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr"/>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr"/>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr"/>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H67" s="4" t="inlineStr"/>
@@ -3000,7 +3000,7 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr"/>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr"/>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr"/>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H71" s="4" t="inlineStr"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr"/>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="G73" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="G74" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr"/>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr"/>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr"/>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr"/>
@@ -3380,7 +3380,7 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr"/>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr"/>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr"/>
@@ -3494,7 +3494,7 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr"/>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="G82" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr"/>
@@ -3570,7 +3570,7 @@
       </c>
       <c r="G83" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr"/>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr"/>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr"/>
@@ -3684,7 +3684,7 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr"/>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="G87" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr"/>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="G88" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr"/>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H89" s="4" t="inlineStr"/>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:39</t>
+          <t>2026-06-24 09:20:41</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr"/>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="G91" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:42</t>
+          <t>2026-06-24 09:20:43</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr"/>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="G92" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr"/>
@@ -3950,7 +3950,7 @@
       </c>
       <c r="G93" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr"/>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr"/>
@@ -4026,7 +4026,7 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H95" s="4" t="inlineStr"/>
@@ -4064,7 +4064,7 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr"/>
@@ -4102,7 +4102,7 @@
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H97" s="4" t="inlineStr"/>
@@ -4140,7 +4140,7 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H98" s="4" t="inlineStr"/>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="G99" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H99" s="4" t="inlineStr"/>
@@ -4216,7 +4216,7 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr"/>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H101" s="4" t="inlineStr"/>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr"/>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H103" s="4" t="inlineStr"/>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H104" s="4" t="inlineStr"/>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H107" s="4" t="inlineStr"/>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr"/>
@@ -4558,7 +4558,7 @@
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr"/>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr"/>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="G111" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H111" s="4" t="inlineStr"/>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H112" s="4" t="inlineStr"/>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="G113" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H113" s="4" t="inlineStr"/>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H114" s="4" t="inlineStr"/>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="G115" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H115" s="4" t="inlineStr"/>
@@ -4824,7 +4824,7 @@
       </c>
       <c r="G116" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H116" s="4" t="inlineStr"/>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H117" s="4" t="inlineStr"/>
@@ -4900,7 +4900,7 @@
       </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H118" s="4" t="inlineStr"/>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="G119" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H119" s="4" t="inlineStr"/>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="G120" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H120" s="4" t="inlineStr"/>
@@ -5014,7 +5014,7 @@
       </c>
       <c r="G121" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H121" s="4" t="inlineStr"/>
@@ -5052,7 +5052,7 @@
       </c>
       <c r="G122" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H122" s="4" t="inlineStr"/>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="G123" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H123" s="4" t="inlineStr"/>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="G124" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H124" s="4" t="inlineStr"/>
@@ -5166,7 +5166,7 @@
       </c>
       <c r="G125" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H125" s="4" t="inlineStr"/>
@@ -5204,7 +5204,7 @@
       </c>
       <c r="G126" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H126" s="4" t="inlineStr"/>
@@ -5242,7 +5242,7 @@
       </c>
       <c r="G127" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H127" s="4" t="inlineStr"/>
@@ -5280,7 +5280,7 @@
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H128" s="4" t="inlineStr"/>
@@ -5318,7 +5318,7 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H129" s="4" t="inlineStr"/>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H130" s="4" t="inlineStr"/>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H131" s="4" t="inlineStr"/>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H132" s="4" t="inlineStr"/>
@@ -5470,7 +5470,7 @@
       </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H133" s="4" t="inlineStr"/>
@@ -5508,7 +5508,7 @@
       </c>
       <c r="G134" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H134" s="4" t="inlineStr"/>
@@ -5546,7 +5546,7 @@
       </c>
       <c r="G135" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H135" s="4" t="inlineStr"/>
@@ -5584,7 +5584,7 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H136" s="4" t="inlineStr"/>
@@ -5622,7 +5622,7 @@
       </c>
       <c r="G137" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H137" s="4" t="inlineStr"/>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="G138" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H138" s="4" t="inlineStr"/>
@@ -5698,7 +5698,7 @@
       </c>
       <c r="G139" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H139" s="4" t="inlineStr"/>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H140" s="4" t="inlineStr"/>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H141" s="4" t="inlineStr"/>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H142" s="4" t="inlineStr"/>
@@ -5850,7 +5850,7 @@
       </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H143" s="4" t="inlineStr"/>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="G144" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H144" s="4" t="inlineStr"/>
@@ -5926,7 +5926,7 @@
       </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H145" s="4" t="inlineStr"/>
@@ -5964,7 +5964,7 @@
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H146" s="4" t="inlineStr"/>
@@ -6002,7 +6002,7 @@
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H147" s="4" t="inlineStr"/>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H148" s="4" t="inlineStr"/>
@@ -6078,7 +6078,7 @@
       </c>
       <c r="G149" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H149" s="4" t="inlineStr"/>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="G150" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H150" s="4" t="inlineStr"/>
@@ -6154,7 +6154,7 @@
       </c>
       <c r="G151" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H151" s="4" t="inlineStr"/>
@@ -6192,7 +6192,7 @@
       </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H152" s="4" t="inlineStr"/>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="G153" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H153" s="4" t="inlineStr"/>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="G154" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H154" s="4" t="inlineStr"/>
@@ -6306,7 +6306,7 @@
       </c>
       <c r="G155" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H155" s="4" t="inlineStr"/>
@@ -6344,7 +6344,7 @@
       </c>
       <c r="G156" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H156" s="4" t="inlineStr"/>
@@ -6382,7 +6382,7 @@
       </c>
       <c r="G157" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H157" s="4" t="inlineStr"/>
@@ -6420,7 +6420,7 @@
       </c>
       <c r="G158" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H158" s="4" t="inlineStr"/>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="G159" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H159" s="4" t="inlineStr"/>
@@ -6496,7 +6496,7 @@
       </c>
       <c r="G160" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H160" s="4" t="inlineStr"/>
@@ -6534,7 +6534,7 @@
       </c>
       <c r="G161" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H161" s="4" t="inlineStr"/>
@@ -6572,7 +6572,7 @@
       </c>
       <c r="G162" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H162" s="4" t="inlineStr"/>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="G163" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H163" s="4" t="inlineStr"/>
@@ -6648,7 +6648,7 @@
       </c>
       <c r="G164" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H164" s="4" t="inlineStr"/>
@@ -6686,7 +6686,7 @@
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H165" s="4" t="inlineStr"/>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="G166" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H166" s="4" t="inlineStr"/>
@@ -6762,7 +6762,7 @@
       </c>
       <c r="G167" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H167" s="4" t="inlineStr"/>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="G168" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H168" s="4" t="inlineStr"/>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="G169" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H169" s="4" t="inlineStr"/>
@@ -6876,7 +6876,7 @@
       </c>
       <c r="G170" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H170" s="4" t="inlineStr"/>
@@ -6914,7 +6914,7 @@
       </c>
       <c r="G171" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H171" s="4" t="inlineStr"/>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="G172" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H172" s="4" t="inlineStr"/>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="G173" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H173" s="4" t="inlineStr"/>
@@ -7028,7 +7028,7 @@
       </c>
       <c r="G174" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H174" s="4" t="inlineStr"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="G175" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H175" s="4" t="inlineStr"/>
@@ -7104,7 +7104,7 @@
       </c>
       <c r="G176" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H176" s="4" t="inlineStr"/>
@@ -7142,7 +7142,7 @@
       </c>
       <c r="G177" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H177" s="4" t="inlineStr"/>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="G178" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H178" s="4" t="inlineStr"/>
@@ -7218,7 +7218,7 @@
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H179" s="4" t="inlineStr"/>
@@ -7256,7 +7256,7 @@
       </c>
       <c r="G180" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H180" s="4" t="inlineStr"/>
@@ -7294,7 +7294,7 @@
       </c>
       <c r="G181" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H181" s="4" t="inlineStr"/>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H182" s="4" t="inlineStr"/>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H183" s="4" t="inlineStr"/>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H184" s="4" t="inlineStr"/>
@@ -7446,7 +7446,7 @@
       </c>
       <c r="G185" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H185" s="4" t="inlineStr"/>
@@ -7484,7 +7484,7 @@
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H186" s="4" t="inlineStr"/>
@@ -7522,7 +7522,7 @@
       </c>
       <c r="G187" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H187" s="4" t="inlineStr"/>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="G188" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H188" s="4" t="inlineStr"/>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="G189" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H189" s="4" t="inlineStr"/>
@@ -7636,7 +7636,7 @@
       </c>
       <c r="G190" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H190" s="4" t="inlineStr"/>
@@ -7674,7 +7674,7 @@
       </c>
       <c r="G191" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H191" s="4" t="inlineStr"/>
@@ -7712,7 +7712,7 @@
       </c>
       <c r="G192" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H192" s="4" t="inlineStr"/>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="G193" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H193" s="4" t="inlineStr"/>
@@ -7788,7 +7788,7 @@
       </c>
       <c r="G194" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H194" s="4" t="inlineStr"/>
@@ -7826,7 +7826,7 @@
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H195" s="4" t="inlineStr"/>
@@ -7864,7 +7864,7 @@
       </c>
       <c r="G196" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H196" s="4" t="inlineStr"/>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="G197" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H197" s="4" t="inlineStr"/>
@@ -7940,7 +7940,7 @@
       </c>
       <c r="G198" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H198" s="4" t="inlineStr"/>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="G199" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H199" s="4" t="inlineStr"/>
@@ -8016,7 +8016,7 @@
       </c>
       <c r="G200" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H200" s="4" t="inlineStr"/>
@@ -8054,7 +8054,7 @@
       </c>
       <c r="G201" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H201" s="4" t="inlineStr"/>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="G202" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H202" s="4" t="inlineStr"/>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="G203" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H203" s="4" t="inlineStr"/>
@@ -8168,7 +8168,7 @@
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H204" s="4" t="inlineStr"/>
@@ -8206,7 +8206,7 @@
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H205" s="4" t="inlineStr"/>
@@ -8244,7 +8244,7 @@
       </c>
       <c r="G206" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H206" s="4" t="inlineStr"/>
@@ -8282,7 +8282,7 @@
       </c>
       <c r="G207" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H207" s="4" t="inlineStr"/>
@@ -8320,7 +8320,7 @@
       </c>
       <c r="G208" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H208" s="4" t="inlineStr"/>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="G209" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H209" s="4" t="inlineStr"/>
@@ -8396,7 +8396,7 @@
       </c>
       <c r="G210" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H210" s="4" t="inlineStr"/>
@@ -8434,7 +8434,7 @@
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H211" s="4" t="inlineStr"/>
@@ -8472,7 +8472,7 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H212" s="4" t="inlineStr"/>
@@ -8510,7 +8510,7 @@
       </c>
       <c r="G213" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H213" s="4" t="inlineStr"/>
@@ -8548,7 +8548,7 @@
       </c>
       <c r="G214" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H214" s="4" t="inlineStr"/>
@@ -8586,7 +8586,7 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H215" s="4" t="inlineStr"/>
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G216" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H216" s="4" t="inlineStr"/>
@@ -8662,7 +8662,7 @@
       </c>
       <c r="G217" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H217" s="4" t="inlineStr"/>
@@ -8700,7 +8700,7 @@
       </c>
       <c r="G218" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H218" s="4" t="inlineStr"/>
@@ -8738,7 +8738,7 @@
       </c>
       <c r="G219" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H219" s="4" t="inlineStr"/>
@@ -8776,7 +8776,7 @@
       </c>
       <c r="G220" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H220" s="4" t="inlineStr"/>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="G221" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H221" s="4" t="inlineStr"/>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="G222" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H222" s="4" t="inlineStr"/>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="G223" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H223" s="4" t="inlineStr"/>
@@ -8928,7 +8928,7 @@
       </c>
       <c r="G224" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H224" s="4" t="inlineStr"/>
@@ -8966,7 +8966,7 @@
       </c>
       <c r="G225" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H225" s="4" t="inlineStr"/>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="G226" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H226" s="4" t="inlineStr"/>
@@ -9042,7 +9042,7 @@
       </c>
       <c r="G227" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H227" s="4" t="inlineStr"/>
@@ -9080,7 +9080,7 @@
       </c>
       <c r="G228" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H228" s="4" t="inlineStr"/>
@@ -9118,7 +9118,7 @@
       </c>
       <c r="G229" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H229" s="4" t="inlineStr"/>
@@ -9156,7 +9156,7 @@
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H230" s="4" t="inlineStr"/>
@@ -9194,7 +9194,7 @@
       </c>
       <c r="G231" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H231" s="4" t="inlineStr"/>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="G232" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H232" s="4" t="inlineStr"/>
@@ -9270,7 +9270,7 @@
       </c>
       <c r="G233" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H233" s="4" t="inlineStr"/>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="G234" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H234" s="4" t="inlineStr"/>
@@ -9346,7 +9346,7 @@
       </c>
       <c r="G235" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H235" s="4" t="inlineStr"/>
@@ -9384,7 +9384,7 @@
       </c>
       <c r="G236" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H236" s="4" t="inlineStr"/>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="G237" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H237" s="4" t="inlineStr"/>
@@ -9460,7 +9460,7 @@
       </c>
       <c r="G238" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H238" s="4" t="inlineStr"/>
@@ -9498,7 +9498,7 @@
       </c>
       <c r="G239" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H239" s="4" t="inlineStr"/>
@@ -9536,7 +9536,7 @@
       </c>
       <c r="G240" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H240" s="4" t="inlineStr"/>
@@ -9574,7 +9574,7 @@
       </c>
       <c r="G241" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H241" s="4" t="inlineStr"/>
@@ -9612,7 +9612,7 @@
       </c>
       <c r="G242" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H242" s="4" t="inlineStr"/>
@@ -9650,7 +9650,7 @@
       </c>
       <c r="G243" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H243" s="4" t="inlineStr"/>
@@ -9688,7 +9688,7 @@
       </c>
       <c r="G244" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H244" s="4" t="inlineStr"/>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="G245" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H245" s="4" t="inlineStr"/>
@@ -9764,7 +9764,7 @@
       </c>
       <c r="G246" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H246" s="4" t="inlineStr"/>
@@ -9802,7 +9802,7 @@
       </c>
       <c r="G247" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H247" s="4" t="inlineStr"/>
@@ -9840,7 +9840,7 @@
       </c>
       <c r="G248" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H248" s="4" t="inlineStr"/>
@@ -9878,7 +9878,7 @@
       </c>
       <c r="G249" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H249" s="4" t="inlineStr"/>
@@ -9916,7 +9916,7 @@
       </c>
       <c r="G250" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H250" s="4" t="inlineStr"/>
@@ -9954,7 +9954,7 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H251" s="4" t="inlineStr"/>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="G252" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H252" s="4" t="inlineStr"/>
@@ -10030,7 +10030,7 @@
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H253" s="4" t="inlineStr"/>
@@ -10068,7 +10068,7 @@
       </c>
       <c r="G254" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H254" s="4" t="inlineStr"/>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H255" s="4" t="inlineStr"/>
@@ -10144,7 +10144,7 @@
       </c>
       <c r="G256" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H256" s="4" t="inlineStr"/>
@@ -10182,7 +10182,7 @@
       </c>
       <c r="G257" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H257" s="4" t="inlineStr"/>
@@ -10220,7 +10220,7 @@
       </c>
       <c r="G258" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H258" s="4" t="inlineStr"/>
@@ -10258,7 +10258,7 @@
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H259" s="4" t="inlineStr"/>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="G260" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H260" s="4" t="inlineStr"/>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="G261" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H261" s="4" t="inlineStr"/>
@@ -10372,7 +10372,7 @@
       </c>
       <c r="G262" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H262" s="4" t="inlineStr"/>
@@ -10410,7 +10410,7 @@
       </c>
       <c r="G263" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H263" s="4" t="inlineStr"/>
@@ -10448,7 +10448,7 @@
       </c>
       <c r="G264" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H264" s="4" t="inlineStr"/>
@@ -10486,7 +10486,7 @@
       </c>
       <c r="G265" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H265" s="4" t="inlineStr"/>
@@ -10524,7 +10524,7 @@
       </c>
       <c r="G266" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H266" s="4" t="inlineStr"/>
@@ -10562,7 +10562,7 @@
       </c>
       <c r="G267" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H267" s="4" t="inlineStr"/>
@@ -10600,7 +10600,7 @@
       </c>
       <c r="G268" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H268" s="4" t="inlineStr"/>
@@ -10638,7 +10638,7 @@
       </c>
       <c r="G269" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H269" s="4" t="inlineStr"/>
@@ -10676,7 +10676,7 @@
       </c>
       <c r="G270" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H270" s="4" t="inlineStr"/>
@@ -10714,7 +10714,7 @@
       </c>
       <c r="G271" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H271" s="4" t="inlineStr"/>
@@ -10752,7 +10752,7 @@
       </c>
       <c r="G272" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H272" s="4" t="inlineStr"/>
@@ -10790,7 +10790,7 @@
       </c>
       <c r="G273" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H273" s="4" t="inlineStr"/>
@@ -10828,7 +10828,7 @@
       </c>
       <c r="G274" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H274" s="4" t="inlineStr"/>
@@ -10866,7 +10866,7 @@
       </c>
       <c r="G275" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H275" s="4" t="inlineStr"/>
@@ -10904,7 +10904,7 @@
       </c>
       <c r="G276" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H276" s="4" t="inlineStr"/>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="G277" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H277" s="4" t="inlineStr"/>
@@ -10980,7 +10980,7 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H278" s="4" t="inlineStr"/>
@@ -11018,7 +11018,7 @@
       </c>
       <c r="G279" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H279" s="4" t="inlineStr"/>
@@ -11056,7 +11056,7 @@
       </c>
       <c r="G280" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H280" s="4" t="inlineStr"/>
@@ -11094,7 +11094,7 @@
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H281" s="4" t="inlineStr"/>
@@ -11132,7 +11132,7 @@
       </c>
       <c r="G282" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H282" s="4" t="inlineStr"/>
@@ -11170,7 +11170,7 @@
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H283" s="4" t="inlineStr"/>
@@ -11208,7 +11208,7 @@
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H284" s="4" t="inlineStr"/>
@@ -11246,7 +11246,7 @@
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H285" s="4" t="inlineStr"/>
@@ -11284,7 +11284,7 @@
       </c>
       <c r="G286" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H286" s="4" t="inlineStr"/>
@@ -11322,7 +11322,7 @@
       </c>
       <c r="G287" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H287" s="4" t="inlineStr"/>
@@ -11360,7 +11360,7 @@
       </c>
       <c r="G288" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H288" s="4" t="inlineStr"/>
@@ -11398,7 +11398,7 @@
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H289" s="4" t="inlineStr"/>
@@ -11436,7 +11436,7 @@
       </c>
       <c r="G290" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H290" s="4" t="inlineStr"/>
@@ -11474,7 +11474,7 @@
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H291" s="4" t="inlineStr"/>
@@ -11512,7 +11512,7 @@
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H292" s="4" t="inlineStr"/>
@@ -11550,7 +11550,7 @@
       </c>
       <c r="G293" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H293" s="4" t="inlineStr"/>
@@ -11588,7 +11588,7 @@
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H294" s="4" t="inlineStr"/>
@@ -11626,7 +11626,7 @@
       </c>
       <c r="G295" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H295" s="4" t="inlineStr"/>
@@ -11664,7 +11664,7 @@
       </c>
       <c r="G296" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H296" s="4" t="inlineStr"/>
@@ -11702,7 +11702,7 @@
       </c>
       <c r="G297" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H297" s="4" t="inlineStr"/>
@@ -11740,7 +11740,7 @@
       </c>
       <c r="G298" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H298" s="4" t="inlineStr"/>
@@ -11778,7 +11778,7 @@
       </c>
       <c r="G299" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H299" s="4" t="inlineStr"/>
@@ -11816,7 +11816,7 @@
       </c>
       <c r="G300" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H300" s="4" t="inlineStr"/>
@@ -11854,7 +11854,7 @@
       </c>
       <c r="G301" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H301" s="4" t="inlineStr"/>
@@ -11892,7 +11892,7 @@
       </c>
       <c r="G302" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H302" s="4" t="inlineStr"/>
@@ -11930,7 +11930,7 @@
       </c>
       <c r="G303" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H303" s="4" t="inlineStr"/>
@@ -11968,7 +11968,7 @@
       </c>
       <c r="G304" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H304" s="4" t="inlineStr"/>
@@ -12006,7 +12006,7 @@
       </c>
       <c r="G305" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H305" s="4" t="inlineStr"/>
@@ -12044,7 +12044,7 @@
       </c>
       <c r="G306" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H306" s="4" t="inlineStr"/>
@@ -12082,7 +12082,7 @@
       </c>
       <c r="G307" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H307" s="4" t="inlineStr"/>
@@ -12120,7 +12120,7 @@
       </c>
       <c r="G308" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H308" s="4" t="inlineStr"/>
@@ -12158,7 +12158,7 @@
       </c>
       <c r="G309" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H309" s="4" t="inlineStr"/>
@@ -12196,7 +12196,7 @@
       </c>
       <c r="G310" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H310" s="4" t="inlineStr"/>
@@ -12234,7 +12234,7 @@
       </c>
       <c r="G311" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H311" s="4" t="inlineStr"/>
@@ -12272,7 +12272,7 @@
       </c>
       <c r="G312" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H312" s="4" t="inlineStr"/>
@@ -12310,7 +12310,7 @@
       </c>
       <c r="G313" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H313" s="4" t="inlineStr"/>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="G314" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H314" s="4" t="inlineStr"/>
@@ -12386,7 +12386,7 @@
       </c>
       <c r="G315" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H315" s="4" t="inlineStr"/>
@@ -12424,7 +12424,7 @@
       </c>
       <c r="G316" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H316" s="4" t="inlineStr"/>
@@ -12462,7 +12462,7 @@
       </c>
       <c r="G317" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H317" s="4" t="inlineStr"/>
@@ -12500,7 +12500,7 @@
       </c>
       <c r="G318" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H318" s="4" t="inlineStr"/>
@@ -12538,7 +12538,7 @@
       </c>
       <c r="G319" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H319" s="4" t="inlineStr"/>
@@ -12576,7 +12576,7 @@
       </c>
       <c r="G320" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H320" s="4" t="inlineStr"/>
@@ -12614,7 +12614,7 @@
       </c>
       <c r="G321" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H321" s="4" t="inlineStr"/>
@@ -12652,7 +12652,7 @@
       </c>
       <c r="G322" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H322" s="4" t="inlineStr"/>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="G323" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H323" s="4" t="inlineStr"/>
@@ -12728,7 +12728,7 @@
       </c>
       <c r="G324" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H324" s="4" t="inlineStr"/>
@@ -12766,7 +12766,7 @@
       </c>
       <c r="G325" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H325" s="4" t="inlineStr"/>
@@ -12804,7 +12804,7 @@
       </c>
       <c r="G326" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H326" s="4" t="inlineStr"/>
@@ -12842,7 +12842,7 @@
       </c>
       <c r="G327" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H327" s="4" t="inlineStr"/>
@@ -12880,7 +12880,7 @@
       </c>
       <c r="G328" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H328" s="4" t="inlineStr"/>
@@ -12918,7 +12918,7 @@
       </c>
       <c r="G329" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H329" s="4" t="inlineStr"/>
@@ -12956,7 +12956,7 @@
       </c>
       <c r="G330" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H330" s="4" t="inlineStr"/>
@@ -12994,7 +12994,7 @@
       </c>
       <c r="G331" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H331" s="4" t="inlineStr"/>
@@ -13032,7 +13032,7 @@
       </c>
       <c r="G332" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H332" s="4" t="inlineStr"/>
@@ -13070,7 +13070,7 @@
       </c>
       <c r="G333" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H333" s="4" t="inlineStr"/>
@@ -13108,7 +13108,7 @@
       </c>
       <c r="G334" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H334" s="4" t="inlineStr"/>
@@ -13146,7 +13146,7 @@
       </c>
       <c r="G335" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H335" s="4" t="inlineStr"/>
@@ -13184,7 +13184,7 @@
       </c>
       <c r="G336" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H336" s="4" t="inlineStr"/>
@@ -13222,7 +13222,7 @@
       </c>
       <c r="G337" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H337" s="4" t="inlineStr"/>
@@ -13260,7 +13260,7 @@
       </c>
       <c r="G338" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H338" s="4" t="inlineStr"/>
@@ -13298,7 +13298,7 @@
       </c>
       <c r="G339" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H339" s="4" t="inlineStr"/>
@@ -13336,7 +13336,7 @@
       </c>
       <c r="G340" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H340" s="4" t="inlineStr"/>
@@ -13374,7 +13374,7 @@
       </c>
       <c r="G341" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H341" s="4" t="inlineStr"/>
@@ -13412,7 +13412,7 @@
       </c>
       <c r="G342" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H342" s="4" t="inlineStr"/>
@@ -13450,7 +13450,7 @@
       </c>
       <c r="G343" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H343" s="4" t="inlineStr"/>
@@ -13488,7 +13488,7 @@
       </c>
       <c r="G344" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H344" s="4" t="inlineStr"/>
@@ -13526,7 +13526,7 @@
       </c>
       <c r="G345" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H345" s="4" t="inlineStr"/>
@@ -13564,7 +13564,7 @@
       </c>
       <c r="G346" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H346" s="4" t="inlineStr"/>
@@ -13602,7 +13602,7 @@
       </c>
       <c r="G347" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H347" s="4" t="inlineStr"/>
@@ -13640,7 +13640,7 @@
       </c>
       <c r="G348" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H348" s="4" t="inlineStr"/>
@@ -13678,7 +13678,7 @@
       </c>
       <c r="G349" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H349" s="4" t="inlineStr"/>
@@ -13716,7 +13716,7 @@
       </c>
       <c r="G350" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H350" s="4" t="inlineStr"/>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="G351" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H351" s="4" t="inlineStr"/>
@@ -13792,7 +13792,7 @@
       </c>
       <c r="G352" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H352" s="4" t="inlineStr"/>
@@ -13830,7 +13830,7 @@
       </c>
       <c r="G353" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H353" s="4" t="inlineStr"/>
@@ -13868,7 +13868,7 @@
       </c>
       <c r="G354" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H354" s="4" t="inlineStr"/>
@@ -13906,7 +13906,7 @@
       </c>
       <c r="G355" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H355" s="4" t="inlineStr"/>
@@ -13944,7 +13944,7 @@
       </c>
       <c r="G356" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H356" s="4" t="inlineStr"/>
@@ -13982,7 +13982,7 @@
       </c>
       <c r="G357" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H357" s="4" t="inlineStr"/>
@@ -14020,7 +14020,7 @@
       </c>
       <c r="G358" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H358" s="4" t="inlineStr"/>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="G359" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H359" s="4" t="inlineStr"/>
@@ -14096,7 +14096,7 @@
       </c>
       <c r="G360" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H360" s="4" t="inlineStr"/>
@@ -14134,7 +14134,7 @@
       </c>
       <c r="G361" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H361" s="4" t="inlineStr"/>
@@ -14172,7 +14172,7 @@
       </c>
       <c r="G362" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H362" s="4" t="inlineStr"/>
@@ -14210,7 +14210,7 @@
       </c>
       <c r="G363" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H363" s="4" t="inlineStr"/>
@@ -14248,7 +14248,7 @@
       </c>
       <c r="G364" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H364" s="4" t="inlineStr"/>
@@ -14286,7 +14286,7 @@
       </c>
       <c r="G365" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H365" s="4" t="inlineStr"/>
@@ -14324,7 +14324,7 @@
       </c>
       <c r="G366" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H366" s="4" t="inlineStr"/>
@@ -14362,7 +14362,7 @@
       </c>
       <c r="G367" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H367" s="4" t="inlineStr"/>
@@ -14400,7 +14400,7 @@
       </c>
       <c r="G368" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H368" s="4" t="inlineStr"/>
@@ -14438,7 +14438,7 @@
       </c>
       <c r="G369" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H369" s="4" t="inlineStr"/>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="G370" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H370" s="4" t="inlineStr"/>
@@ -14514,7 +14514,7 @@
       </c>
       <c r="G371" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H371" s="4" t="inlineStr"/>
@@ -14552,7 +14552,7 @@
       </c>
       <c r="G372" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H372" s="4" t="inlineStr"/>
@@ -14590,7 +14590,7 @@
       </c>
       <c r="G373" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H373" s="4" t="inlineStr"/>
@@ -14628,7 +14628,7 @@
       </c>
       <c r="G374" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H374" s="4" t="inlineStr"/>
@@ -14666,7 +14666,7 @@
       </c>
       <c r="G375" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H375" s="4" t="inlineStr"/>
@@ -14704,7 +14704,7 @@
       </c>
       <c r="G376" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H376" s="4" t="inlineStr"/>
@@ -14742,7 +14742,7 @@
       </c>
       <c r="G377" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H377" s="4" t="inlineStr"/>
@@ -14780,7 +14780,7 @@
       </c>
       <c r="G378" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H378" s="4" t="inlineStr"/>
@@ -14818,7 +14818,7 @@
       </c>
       <c r="G379" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H379" s="4" t="inlineStr"/>
@@ -14856,7 +14856,7 @@
       </c>
       <c r="G380" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H380" s="4" t="inlineStr"/>
@@ -14894,7 +14894,7 @@
       </c>
       <c r="G381" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H381" s="4" t="inlineStr"/>
@@ -14932,7 +14932,7 @@
       </c>
       <c r="G382" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H382" s="4" t="inlineStr"/>
@@ -14970,7 +14970,7 @@
       </c>
       <c r="G383" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H383" s="4" t="inlineStr"/>
@@ -15008,7 +15008,7 @@
       </c>
       <c r="G384" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H384" s="4" t="inlineStr"/>
@@ -15046,7 +15046,7 @@
       </c>
       <c r="G385" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H385" s="4" t="inlineStr"/>
@@ -15084,7 +15084,7 @@
       </c>
       <c r="G386" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H386" s="4" t="inlineStr"/>
@@ -15122,7 +15122,7 @@
       </c>
       <c r="G387" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H387" s="4" t="inlineStr"/>
@@ -15160,7 +15160,7 @@
       </c>
       <c r="G388" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H388" s="4" t="inlineStr"/>
@@ -15198,7 +15198,7 @@
       </c>
       <c r="G389" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H389" s="4" t="inlineStr"/>
@@ -15236,7 +15236,7 @@
       </c>
       <c r="G390" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H390" s="4" t="inlineStr"/>
@@ -15274,7 +15274,7 @@
       </c>
       <c r="G391" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H391" s="4" t="inlineStr"/>
@@ -15312,7 +15312,7 @@
       </c>
       <c r="G392" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H392" s="4" t="inlineStr"/>
@@ -15350,7 +15350,7 @@
       </c>
       <c r="G393" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H393" s="4" t="inlineStr"/>
@@ -15388,7 +15388,7 @@
       </c>
       <c r="G394" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H394" s="4" t="inlineStr"/>
@@ -15426,7 +15426,7 @@
       </c>
       <c r="G395" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H395" s="4" t="inlineStr"/>
@@ -15464,7 +15464,7 @@
       </c>
       <c r="G396" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H396" s="4" t="inlineStr"/>
@@ -15502,7 +15502,7 @@
       </c>
       <c r="G397" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H397" s="4" t="inlineStr"/>
@@ -15540,7 +15540,7 @@
       </c>
       <c r="G398" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H398" s="4" t="inlineStr"/>
@@ -15578,7 +15578,7 @@
       </c>
       <c r="G399" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H399" s="4" t="inlineStr"/>
@@ -15616,7 +15616,7 @@
       </c>
       <c r="G400" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H400" s="4" t="inlineStr"/>
@@ -15654,7 +15654,7 @@
       </c>
       <c r="G401" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H401" s="4" t="inlineStr"/>
@@ -15692,7 +15692,7 @@
       </c>
       <c r="G402" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H402" s="4" t="inlineStr"/>
@@ -15730,7 +15730,7 @@
       </c>
       <c r="G403" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H403" s="4" t="inlineStr"/>
@@ -15768,7 +15768,7 @@
       </c>
       <c r="G404" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H404" s="4" t="inlineStr"/>
@@ -15806,7 +15806,7 @@
       </c>
       <c r="G405" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H405" s="4" t="inlineStr"/>
@@ -15844,7 +15844,7 @@
       </c>
       <c r="G406" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H406" s="4" t="inlineStr"/>
@@ -15882,7 +15882,7 @@
       </c>
       <c r="G407" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H407" s="4" t="inlineStr"/>
@@ -15920,7 +15920,7 @@
       </c>
       <c r="G408" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H408" s="4" t="inlineStr"/>
@@ -15958,7 +15958,7 @@
       </c>
       <c r="G409" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H409" s="4" t="inlineStr"/>
@@ -15996,7 +15996,7 @@
       </c>
       <c r="G410" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H410" s="4" t="inlineStr"/>
@@ -16034,7 +16034,7 @@
       </c>
       <c r="G411" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H411" s="4" t="inlineStr"/>
@@ -16072,7 +16072,7 @@
       </c>
       <c r="G412" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H412" s="4" t="inlineStr"/>
@@ -16110,7 +16110,7 @@
       </c>
       <c r="G413" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H413" s="4" t="inlineStr"/>
@@ -16148,7 +16148,7 @@
       </c>
       <c r="G414" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H414" s="4" t="inlineStr"/>
@@ -16186,7 +16186,7 @@
       </c>
       <c r="G415" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H415" s="4" t="inlineStr"/>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="G416" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H416" s="4" t="inlineStr"/>
@@ -16262,7 +16262,7 @@
       </c>
       <c r="G417" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H417" s="4" t="inlineStr"/>
@@ -16300,7 +16300,7 @@
       </c>
       <c r="G418" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H418" s="4" t="inlineStr"/>
@@ -16338,7 +16338,7 @@
       </c>
       <c r="G419" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H419" s="4" t="inlineStr"/>
@@ -16376,7 +16376,7 @@
       </c>
       <c r="G420" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H420" s="4" t="inlineStr"/>
@@ -16414,7 +16414,7 @@
       </c>
       <c r="G421" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H421" s="4" t="inlineStr"/>
@@ -16452,7 +16452,7 @@
       </c>
       <c r="G422" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H422" s="4" t="inlineStr"/>
@@ -16490,7 +16490,7 @@
       </c>
       <c r="G423" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H423" s="4" t="inlineStr"/>
@@ -16528,7 +16528,7 @@
       </c>
       <c r="G424" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H424" s="4" t="inlineStr"/>
@@ -16566,7 +16566,7 @@
       </c>
       <c r="G425" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H425" s="4" t="inlineStr"/>
@@ -16604,7 +16604,7 @@
       </c>
       <c r="G426" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H426" s="4" t="inlineStr"/>
@@ -16642,7 +16642,7 @@
       </c>
       <c r="G427" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H427" s="4" t="inlineStr"/>
@@ -16680,7 +16680,7 @@
       </c>
       <c r="G428" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H428" s="4" t="inlineStr"/>
@@ -16718,7 +16718,7 @@
       </c>
       <c r="G429" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H429" s="4" t="inlineStr"/>
@@ -16756,7 +16756,7 @@
       </c>
       <c r="G430" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H430" s="4" t="inlineStr"/>
@@ -16794,7 +16794,7 @@
       </c>
       <c r="G431" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H431" s="4" t="inlineStr"/>
@@ -16832,7 +16832,7 @@
       </c>
       <c r="G432" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H432" s="4" t="inlineStr"/>
@@ -16870,7 +16870,7 @@
       </c>
       <c r="G433" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H433" s="4" t="inlineStr"/>
@@ -16908,7 +16908,7 @@
       </c>
       <c r="G434" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H434" s="4" t="inlineStr"/>
@@ -16946,7 +16946,7 @@
       </c>
       <c r="G435" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H435" s="4" t="inlineStr"/>
@@ -16984,7 +16984,7 @@
       </c>
       <c r="G436" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H436" s="4" t="inlineStr"/>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="G437" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H437" s="4" t="inlineStr"/>
@@ -17060,7 +17060,7 @@
       </c>
       <c r="G438" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H438" s="4" t="inlineStr"/>
@@ -17098,7 +17098,7 @@
       </c>
       <c r="G439" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H439" s="4" t="inlineStr"/>
@@ -17136,7 +17136,7 @@
       </c>
       <c r="G440" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H440" s="4" t="inlineStr"/>
@@ -17174,7 +17174,7 @@
       </c>
       <c r="G441" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H441" s="4" t="inlineStr"/>
@@ -17212,7 +17212,7 @@
       </c>
       <c r="G442" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H442" s="4" t="inlineStr"/>
@@ -17250,7 +17250,7 @@
       </c>
       <c r="G443" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H443" s="4" t="inlineStr"/>
@@ -17288,7 +17288,7 @@
       </c>
       <c r="G444" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H444" s="4" t="inlineStr"/>
@@ -17326,7 +17326,7 @@
       </c>
       <c r="G445" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H445" s="4" t="inlineStr"/>
@@ -17364,7 +17364,7 @@
       </c>
       <c r="G446" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H446" s="4" t="inlineStr"/>
@@ -17402,7 +17402,7 @@
       </c>
       <c r="G447" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H447" s="4" t="inlineStr"/>
@@ -17440,7 +17440,7 @@
       </c>
       <c r="G448" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H448" s="4" t="inlineStr"/>
@@ -17478,7 +17478,7 @@
       </c>
       <c r="G449" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H449" s="4" t="inlineStr"/>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="G450" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H450" s="4" t="inlineStr"/>
@@ -17554,7 +17554,7 @@
       </c>
       <c r="G451" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H451" s="4" t="inlineStr"/>
@@ -17592,7 +17592,7 @@
       </c>
       <c r="G452" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H452" s="4" t="inlineStr"/>
@@ -17630,7 +17630,7 @@
       </c>
       <c r="G453" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H453" s="4" t="inlineStr"/>
@@ -17668,7 +17668,7 @@
       </c>
       <c r="G454" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H454" s="4" t="inlineStr"/>
@@ -17706,7 +17706,7 @@
       </c>
       <c r="G455" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H455" s="4" t="inlineStr"/>
@@ -17744,7 +17744,7 @@
       </c>
       <c r="G456" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H456" s="4" t="inlineStr"/>
@@ -17782,7 +17782,7 @@
       </c>
       <c r="G457" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H457" s="4" t="inlineStr"/>
@@ -17820,7 +17820,7 @@
       </c>
       <c r="G458" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H458" s="4" t="inlineStr"/>
@@ -17858,7 +17858,7 @@
       </c>
       <c r="G459" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H459" s="4" t="inlineStr"/>
@@ -17896,7 +17896,7 @@
       </c>
       <c r="G460" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H460" s="4" t="inlineStr"/>
@@ -17934,7 +17934,7 @@
       </c>
       <c r="G461" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H461" s="4" t="inlineStr"/>
@@ -17972,7 +17972,7 @@
       </c>
       <c r="G462" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H462" s="4" t="inlineStr"/>
@@ -18010,7 +18010,7 @@
       </c>
       <c r="G463" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H463" s="4" t="inlineStr"/>
@@ -18048,7 +18048,7 @@
       </c>
       <c r="G464" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H464" s="4" t="inlineStr"/>
@@ -18086,7 +18086,7 @@
       </c>
       <c r="G465" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H465" s="4" t="inlineStr"/>
@@ -18124,7 +18124,7 @@
       </c>
       <c r="G466" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H466" s="4" t="inlineStr"/>
@@ -18162,7 +18162,7 @@
       </c>
       <c r="G467" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H467" s="4" t="inlineStr"/>
@@ -18200,7 +18200,7 @@
       </c>
       <c r="G468" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H468" s="4" t="inlineStr"/>
@@ -18238,7 +18238,7 @@
       </c>
       <c r="G469" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H469" s="4" t="inlineStr"/>
@@ -18276,7 +18276,7 @@
       </c>
       <c r="G470" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H470" s="4" t="inlineStr"/>
@@ -18314,7 +18314,7 @@
       </c>
       <c r="G471" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H471" s="4" t="inlineStr"/>
@@ -18352,7 +18352,7 @@
       </c>
       <c r="G472" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H472" s="4" t="inlineStr"/>
@@ -18390,7 +18390,7 @@
       </c>
       <c r="G473" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H473" s="4" t="inlineStr"/>
@@ -18428,7 +18428,7 @@
       </c>
       <c r="G474" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H474" s="4" t="inlineStr"/>
@@ -18466,7 +18466,7 @@
       </c>
       <c r="G475" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H475" s="4" t="inlineStr"/>
@@ -18504,7 +18504,7 @@
       </c>
       <c r="G476" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H476" s="4" t="inlineStr"/>
@@ -18542,7 +18542,7 @@
       </c>
       <c r="G477" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H477" s="4" t="inlineStr"/>
@@ -18580,7 +18580,7 @@
       </c>
       <c r="G478" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H478" s="4" t="inlineStr"/>
@@ -18618,7 +18618,7 @@
       </c>
       <c r="G479" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 09:12:44</t>
+          <t>2026-06-24 09:20:45</t>
         </is>
       </c>
       <c r="H479" s="4" t="inlineStr"/>

</xml_diff>